<commit_message>
Category Keywords Rule Integration - Implementation Plan
Implementation completed
</commit_message>
<xml_diff>
--- a/Data-Normalization/Data Example/big data.xlsx
+++ b/Data-Normalization/Data Example/big data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Finance-Project\Data-Normalization\Data Example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA717A9-6438-472C-9A87-D94492515F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDEB382-DC56-4BBD-9E77-55B0986FC04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="23280" windowHeight="12480" xr2:uid="{4CA62BB2-8104-49F2-BC93-4318D9023633}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="12">
   <si>
     <t>商户</t>
   </si>
@@ -41,6 +41,21 @@
   </si>
   <si>
     <t>Indomaret</t>
+  </si>
+  <si>
+    <t>cafepoint</t>
+  </si>
+  <si>
+    <t>grab bcs</t>
+  </si>
+  <si>
+    <t>bluebirdtaxi</t>
+  </si>
+  <si>
+    <t>iuran bpjs</t>
+  </si>
+  <si>
+    <t>bus angkot</t>
   </si>
 </sst>
 </file>
@@ -1105,6 +1120,9 @@
       <c r="D7" t="s">
         <v>6</v>
       </c>
+      <c r="E7">
+        <v>45000</v>
+      </c>
       <c r="F7">
         <v>45000</v>
       </c>
@@ -1120,9 +1138,12 @@
         <v>45900</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8">
+        <v>45000</v>
+      </c>
+      <c r="F8">
         <v>45000</v>
       </c>
     </row>
@@ -1137,7 +1158,7 @@
         <v>45900</v>
       </c>
       <c r="D9" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E9">
         <v>45000</v>
@@ -1157,7 +1178,7 @@
         <v>45900</v>
       </c>
       <c r="D10" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E10">
         <v>45000</v>
@@ -1187,7 +1208,7 @@
         <v>45900</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E13">
         <v>45000</v>
@@ -1227,7 +1248,7 @@
         <v>45900</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E15">
         <v>45000</v>

</xml_diff>